<commit_message>
updated path to generic path
</commit_message>
<xml_diff>
--- a/Scripts/Compare 856 with POFR/nonexist.xlsx
+++ b/Scripts/Compare 856 with POFR/nonexist.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,7 +439,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1786252</t>
+          <t>1777268</t>
         </is>
       </c>
     </row>
@@ -449,7 +449,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1794326</t>
+          <t>1780224</t>
         </is>
       </c>
     </row>
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1797247</t>
+          <t>1781809</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1798188</t>
+          <t>1788275</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1798559</t>
+          <t>1789577</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1799470</t>
+          <t>1791219</t>
         </is>
       </c>
     </row>
@@ -499,7 +499,707 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1800057</t>
+          <t>1793364</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1793412</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1793420</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1793507</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1793970</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1794907</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1795546</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1795714</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1796036</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1796425</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1796533</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1796550</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1796559</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1797221</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1797417</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1798613</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1798775</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1798804</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1798956</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1799317</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1799603</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1799678</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1799718</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1799793</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1799846</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1800120</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1800193</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1800237</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1800262</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1800372</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1800383</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1800477</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1800592</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1800911</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1801165</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1801201</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1801209</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1801357</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1801387</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1801814</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1801837</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1801849</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1801947</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1802367</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1802459</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1802469</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1802479</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1802669</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1802687</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1802695</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1802742</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1802748</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1802757</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1803094</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1803244</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1803252</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1803298</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1803390</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1803412</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1803670</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1803709</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1803716</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1803734</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2092426</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2092444</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2092483</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2092486</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2092542</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2092653</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2092668</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2092754</t>
         </is>
       </c>
     </row>

</xml_diff>